<commit_message>
Change logic to seperate module to make quote without registering new item
</commit_message>
<xml_diff>
--- a/Example PL.xlsx
+++ b/Example PL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acsolutions-my.sharepoint.com/personal/niels_ac-solutions_be/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\niels\VSC_Projects\Custom-Odoo\odoo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{7F390DC7-1216-4287-9792-48B3F638E458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFFF5743-1B15-4860-8F7F-6F85CD126E9D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DD5759-A4A2-48AF-8BCA-72987A7A4A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0175591F-D8A5-4571-8C6F-C92C3EBD14E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0175591F-D8A5-4571-8C6F-C92C3EBD14E9}"/>
   </bookViews>
   <sheets>
     <sheet name="QUOTE" sheetId="3" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="107">
   <si>
     <t>Application</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -412,6 +412,31 @@
   <si>
     <t xml:space="preserve">OD 3.7mm 3*0.2mm², PVC/PVC (Black,blue,Red) </t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z409BG</t>
+  </si>
+  <si>
+    <t>Z509BG</t>
+  </si>
+  <si>
+    <t>Z609BG</t>
+  </si>
+  <si>
+    <t>Z209BM</t>
+  </si>
+  <si>
+    <t>Z309BM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z409BM</t>
+  </si>
+  <si>
+    <t>Z509BM</t>
+  </si>
+  <si>
+    <t>Z609BM</t>
   </si>
 </sst>
 </file>
@@ -1157,7 +1182,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1610,6 +1635,12 @@
     <xf numFmtId="169" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="18" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1650,11 +1681,8 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="18" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1662,7 +1690,17 @@
     <cellStyle name="Komma 2" xfId="2" xr:uid="{CF877343-7E00-44C8-89FB-F4DA51A7E72B}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C6500"/>
@@ -2199,23 +2237,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E83C851D-9B41-4F03-90BD-D7886FE835FF}">
   <dimension ref="A1:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="15" width="15.140625" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" customWidth="1"/>
+    <col min="11" max="15" width="15.109375" customWidth="1"/>
+    <col min="16" max="16" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="20" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="20" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C1" s="21"/>
       <c r="M1" s="21"/>
       <c r="N1" s="21"/>
     </row>
-    <row r="2" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="22"/>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
@@ -2236,7 +2274,7 @@
       <c r="P2" s="22"/>
       <c r="Q2" s="22"/>
     </row>
-    <row r="3" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22"/>
       <c r="B3" s="22"/>
       <c r="C3" s="26" t="s">
@@ -2271,7 +2309,7 @@
       <c r="P3" s="22"/>
       <c r="Q3" s="22"/>
     </row>
-    <row r="4" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="22"/>
       <c r="B4" s="22"/>
       <c r="C4" s="29" t="s">
@@ -2287,7 +2325,7 @@
       <c r="G4" s="32">
         <v>10</v>
       </c>
-      <c r="H4" s="146">
+      <c r="H4" s="136">
         <v>1.4</v>
       </c>
       <c r="I4" s="33">
@@ -2306,7 +2344,7 @@
       <c r="P4" s="22"/>
       <c r="Q4" s="22"/>
     </row>
-    <row r="5" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="22"/>
       <c r="B5" s="22"/>
       <c r="C5" s="29" t="s">
@@ -2322,7 +2360,7 @@
       <c r="G5" s="32">
         <v>50</v>
       </c>
-      <c r="H5" s="146">
+      <c r="H5" s="136">
         <v>1.2</v>
       </c>
       <c r="I5" s="33">
@@ -2341,7 +2379,7 @@
       <c r="P5" s="22"/>
       <c r="Q5" s="22"/>
     </row>
-    <row r="6" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="22"/>
       <c r="B6" s="22"/>
       <c r="C6" s="29" t="s">
@@ -2357,7 +2395,7 @@
       <c r="G6" s="32">
         <v>300</v>
       </c>
-      <c r="H6" s="146">
+      <c r="H6" s="136">
         <v>1</v>
       </c>
       <c r="I6" s="33">
@@ -2376,7 +2414,7 @@
       <c r="P6" s="22"/>
       <c r="Q6" s="22"/>
     </row>
-    <row r="7" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="22"/>
       <c r="B7" s="22"/>
       <c r="C7" s="29" t="s">
@@ -2392,7 +2430,7 @@
       <c r="G7" s="32">
         <v>1000</v>
       </c>
-      <c r="H7" s="146">
+      <c r="H7" s="136">
         <v>0.98</v>
       </c>
       <c r="I7" s="33">
@@ -2411,7 +2449,7 @@
       <c r="P7" s="22"/>
       <c r="Q7" s="22"/>
     </row>
-    <row r="8" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="22"/>
       <c r="B8" s="22"/>
       <c r="C8" s="29" t="s">
@@ -2427,7 +2465,7 @@
       <c r="G8" s="32">
         <v>5000</v>
       </c>
-      <c r="H8" s="146">
+      <c r="H8" s="136">
         <v>0.95</v>
       </c>
       <c r="I8" s="33">
@@ -2446,7 +2484,7 @@
       <c r="P8" s="22"/>
       <c r="Q8" s="22"/>
     </row>
-    <row r="9" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22"/>
       <c r="B9" s="22"/>
       <c r="C9" s="29" t="s">
@@ -2462,7 +2500,7 @@
       <c r="G9" s="32">
         <v>10000</v>
       </c>
-      <c r="H9" s="146">
+      <c r="H9" s="136">
         <v>0.9</v>
       </c>
       <c r="I9" s="33">
@@ -2481,7 +2519,7 @@
       <c r="P9" s="22"/>
       <c r="Q9" s="22"/>
     </row>
-    <row r="10" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="29" t="s">
@@ -2497,7 +2535,7 @@
       <c r="G10" s="32">
         <v>20000</v>
       </c>
-      <c r="H10" s="146">
+      <c r="H10" s="136">
         <v>0.88</v>
       </c>
       <c r="I10" s="33">
@@ -2516,7 +2554,7 @@
       <c r="P10" s="22"/>
       <c r="Q10" s="22"/>
     </row>
-    <row r="11" spans="1:17" s="21" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" s="21" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="29" t="s">
@@ -2532,7 +2570,7 @@
       <c r="G11" s="35">
         <v>50000</v>
       </c>
-      <c r="H11" s="147">
+      <c r="H11" s="137">
         <v>0.85</v>
       </c>
       <c r="I11" s="36">
@@ -2551,7 +2589,7 @@
       <c r="P11" s="37"/>
       <c r="Q11" s="22"/>
     </row>
-    <row r="12" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22"/>
       <c r="B12" s="22"/>
       <c r="C12" s="26" t="s">
@@ -2576,99 +2614,99 @@
       </c>
       <c r="Q12" s="22"/>
     </row>
-    <row r="13" spans="1:17" s="20" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" s="20" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C13" s="21"/>
       <c r="E13" s="40"/>
       <c r="M13" s="21"/>
       <c r="N13" s="21"/>
       <c r="P13" s="41"/>
     </row>
-    <row r="14" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C14" s="43"/>
-      <c r="D14" s="136" t="s">
+      <c r="D14" s="138" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="137"/>
-      <c r="F14" s="137"/>
-      <c r="G14" s="137"/>
-      <c r="H14" s="137"/>
-      <c r="I14" s="137"/>
-      <c r="J14" s="137"/>
-      <c r="K14" s="137"/>
-      <c r="L14" s="137"/>
-      <c r="M14" s="138"/>
-      <c r="N14" s="138"/>
-      <c r="O14" s="138"/>
+      <c r="E14" s="139"/>
+      <c r="F14" s="139"/>
+      <c r="G14" s="139"/>
+      <c r="H14" s="139"/>
+      <c r="I14" s="139"/>
+      <c r="J14" s="139"/>
+      <c r="K14" s="139"/>
+      <c r="L14" s="139"/>
+      <c r="M14" s="140"/>
+      <c r="N14" s="140"/>
+      <c r="O14" s="140"/>
       <c r="P14" s="44" t="s">
         <v>50</v>
       </c>
       <c r="Q14" s="45"/>
     </row>
-    <row r="15" spans="1:17" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C15" s="43"/>
       <c r="D15" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="139"/>
-      <c r="F15" s="139"/>
-      <c r="G15" s="139"/>
-      <c r="H15" s="139"/>
-      <c r="I15" s="139"/>
-      <c r="J15" s="139"/>
-      <c r="K15" s="139"/>
-      <c r="L15" s="139"/>
-      <c r="M15" s="140"/>
-      <c r="N15" s="140"/>
-      <c r="O15" s="140"/>
+      <c r="E15" s="141"/>
+      <c r="F15" s="141"/>
+      <c r="G15" s="141"/>
+      <c r="H15" s="141"/>
+      <c r="I15" s="141"/>
+      <c r="J15" s="141"/>
+      <c r="K15" s="141"/>
+      <c r="L15" s="141"/>
+      <c r="M15" s="142"/>
+      <c r="N15" s="142"/>
+      <c r="O15" s="142"/>
       <c r="P15" s="47" t="s">
         <v>52</v>
       </c>
       <c r="Q15" s="48"/>
     </row>
-    <row r="16" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C16" s="43"/>
       <c r="D16" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="140"/>
-      <c r="F16" s="141"/>
-      <c r="G16" s="141"/>
-      <c r="H16" s="141"/>
-      <c r="I16" s="141"/>
-      <c r="J16" s="141"/>
-      <c r="K16" s="141"/>
-      <c r="L16" s="141"/>
-      <c r="M16" s="141"/>
-      <c r="N16" s="141"/>
-      <c r="O16" s="142"/>
+      <c r="E16" s="142"/>
+      <c r="F16" s="143"/>
+      <c r="G16" s="143"/>
+      <c r="H16" s="143"/>
+      <c r="I16" s="143"/>
+      <c r="J16" s="143"/>
+      <c r="K16" s="143"/>
+      <c r="L16" s="143"/>
+      <c r="M16" s="143"/>
+      <c r="N16" s="143"/>
+      <c r="O16" s="144"/>
       <c r="P16" s="49" t="s">
         <v>54</v>
       </c>
       <c r="Q16" s="48"/>
     </row>
-    <row r="17" spans="2:17" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:17" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C17" s="43"/>
       <c r="D17" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="143"/>
-      <c r="F17" s="143"/>
-      <c r="G17" s="143"/>
-      <c r="H17" s="143"/>
-      <c r="I17" s="143"/>
-      <c r="J17" s="143"/>
-      <c r="K17" s="143"/>
-      <c r="L17" s="143"/>
-      <c r="M17" s="144"/>
-      <c r="N17" s="144"/>
-      <c r="O17" s="144"/>
+      <c r="E17" s="145"/>
+      <c r="F17" s="145"/>
+      <c r="G17" s="145"/>
+      <c r="H17" s="145"/>
+      <c r="I17" s="145"/>
+      <c r="J17" s="145"/>
+      <c r="K17" s="145"/>
+      <c r="L17" s="145"/>
+      <c r="M17" s="146"/>
+      <c r="N17" s="146"/>
+      <c r="O17" s="146"/>
       <c r="P17" s="51"/>
       <c r="Q17" s="52" t="str" cm="1">
         <f t="array" ref="Q17">IF(P17&lt;&gt;"",Lastmodified(P17),"")</f>
         <v/>
       </c>
     </row>
-    <row r="18" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C18" s="43"/>
       <c r="D18" s="53"/>
       <c r="E18" s="54"/>
@@ -2683,7 +2721,7 @@
       <c r="N18" s="56"/>
       <c r="O18" s="57"/>
     </row>
-    <row r="19" spans="2:17" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:17" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C19" s="43"/>
       <c r="D19" s="53"/>
       <c r="E19" s="54"/>
@@ -2698,7 +2736,7 @@
       <c r="N19" s="56"/>
       <c r="O19" s="57"/>
     </row>
-    <row r="20" spans="2:17" s="42" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:17" s="42" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="58"/>
       <c r="C20" s="59"/>
       <c r="D20" s="60"/>
@@ -2721,7 +2759,7 @@
       <c r="O20" s="64"/>
       <c r="P20" s="65"/>
     </row>
-    <row r="21" spans="2:17" s="42" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:17" s="42" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="66" t="s">
         <v>58</v>
       </c>
@@ -2770,7 +2808,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B22" s="66" t="s">
         <v>66</v>
       </c>
@@ -2815,7 +2853,7 @@
       </c>
       <c r="P22" s="87"/>
     </row>
-    <row r="23" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="66" t="s">
         <v>67</v>
       </c>
@@ -2854,7 +2892,7 @@
       </c>
       <c r="P23" s="87"/>
     </row>
-    <row r="24" spans="2:17" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:17" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="66"/>
       <c r="C24" s="67" t="s">
         <v>42</v>
@@ -2891,7 +2929,7 @@
       </c>
       <c r="P24" s="87"/>
     </row>
-    <row r="25" spans="2:17" s="42" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:17" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="66"/>
       <c r="C25" s="67" t="s">
         <v>43</v>
@@ -2930,7 +2968,7 @@
       </c>
       <c r="P25" s="87"/>
     </row>
-    <row r="26" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B26" s="66"/>
       <c r="C26" s="67" t="s">
         <v>44</v>
@@ -2967,7 +3005,7 @@
       </c>
       <c r="P26" s="87"/>
     </row>
-    <row r="27" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B27" s="66"/>
       <c r="C27" s="67" t="s">
         <v>45</v>
@@ -3004,7 +3042,7 @@
       </c>
       <c r="P27" s="87"/>
     </row>
-    <row r="28" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B28" s="66"/>
       <c r="C28" s="67" t="s">
         <v>46</v>
@@ -3041,7 +3079,7 @@
       </c>
       <c r="P28" s="87"/>
     </row>
-    <row r="29" spans="2:17" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:17" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="95"/>
       <c r="C29" s="96" t="s">
         <v>47</v>
@@ -3078,7 +3116,7 @@
       </c>
       <c r="P29" s="104"/>
     </row>
-    <row r="30" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="123"/>
       <c r="C30" s="124"/>
       <c r="D30" s="89"/>
@@ -3092,27 +3130,27 @@
       <c r="N30" s="127"/>
       <c r="O30" s="128"/>
     </row>
-    <row r="31" spans="2:17" s="42" customFormat="1" ht="24" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:17" s="42" customFormat="1" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B31" s="123"/>
       <c r="C31" s="124"/>
-      <c r="D31" s="145" t="s">
+      <c r="D31" s="147" t="s">
         <v>88</v>
       </c>
-      <c r="E31" s="145"/>
-      <c r="F31" s="145"/>
-      <c r="G31" s="145"/>
-      <c r="H31" s="145"/>
-      <c r="I31" s="145"/>
-      <c r="J31" s="145"/>
-      <c r="K31" s="145"/>
-      <c r="L31" s="145"/>
-      <c r="M31" s="145"/>
-      <c r="N31" s="145"/>
-      <c r="O31" s="145"/>
-      <c r="P31" s="145"/>
-    </row>
-    <row r="32" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="2:16" s="42" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E31" s="147"/>
+      <c r="F31" s="147"/>
+      <c r="G31" s="147"/>
+      <c r="H31" s="147"/>
+      <c r="I31" s="147"/>
+      <c r="J31" s="147"/>
+      <c r="K31" s="147"/>
+      <c r="L31" s="147"/>
+      <c r="M31" s="147"/>
+      <c r="N31" s="147"/>
+      <c r="O31" s="147"/>
+      <c r="P31" s="147"/>
+    </row>
+    <row r="32" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="33" spans="2:16" s="42" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="58"/>
       <c r="C33" s="59"/>
       <c r="D33" s="60"/>
@@ -3135,7 +3173,7 @@
       <c r="O33" s="64"/>
       <c r="P33" s="65"/>
     </row>
-    <row r="34" spans="2:16" s="42" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:16" s="42" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="66" t="s">
         <v>58</v>
       </c>
@@ -3184,7 +3222,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B35" s="66" t="s">
         <v>66</v>
       </c>
@@ -3235,7 +3273,7 @@
       </c>
       <c r="P35" s="87"/>
     </row>
-    <row r="36" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B36" s="66" t="s">
         <v>67</v>
       </c>
@@ -3269,12 +3307,12 @@
         <v>102</v>
       </c>
       <c r="O36" s="91">
-        <f t="shared" ref="O35:O42" si="5">IF($P$17="",IF(VLOOKUP(C36,$C$4:$E$11,2,FALSE)&gt;$D$12,ROUND(M36,2)&amp;" &gt; Get approval",M36),M36)</f>
+        <f t="shared" ref="O36:O42" si="5">IF($P$17="",IF(VLOOKUP(C36,$C$4:$E$11,2,FALSE)&gt;$D$12,ROUND(M36,2)&amp;" &gt; Get approval",M36),M36)</f>
         <v>2.04</v>
       </c>
       <c r="P36" s="87"/>
     </row>
-    <row r="37" spans="2:16" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:16" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="66"/>
       <c r="C37" s="67" t="s">
         <v>42</v>
@@ -3311,7 +3349,7 @@
       </c>
       <c r="P37" s="87"/>
     </row>
-    <row r="38" spans="2:16" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:16" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="66"/>
       <c r="C38" s="67" t="s">
         <v>43</v>
@@ -3350,7 +3388,7 @@
       </c>
       <c r="P38" s="87"/>
     </row>
-    <row r="39" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B39" s="66"/>
       <c r="C39" s="67" t="s">
         <v>44</v>
@@ -3387,7 +3425,7 @@
       </c>
       <c r="P39" s="87"/>
     </row>
-    <row r="40" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B40" s="66"/>
       <c r="C40" s="67" t="s">
         <v>45</v>
@@ -3424,7 +3462,7 @@
       </c>
       <c r="P40" s="87"/>
     </row>
-    <row r="41" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:16" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B41" s="66"/>
       <c r="C41" s="67" t="s">
         <v>46</v>
@@ -3461,7 +3499,7 @@
       </c>
       <c r="P41" s="87"/>
     </row>
-    <row r="42" spans="2:16" s="42" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:16" s="42" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="95"/>
       <c r="C42" s="96" t="s">
         <v>47</v>
@@ -3507,71 +3545,71 @@
     <mergeCell ref="D31:P31"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:P1">
-    <cfRule type="expression" dxfId="23" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="24" priority="10" stopIfTrue="1">
       <formula>N("_PMRH")=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4:D11">
-    <cfRule type="cellIs" dxfId="22" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="16" operator="greaterThan">
       <formula>$D$12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E4:E11">
-    <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="get approval">
+    <cfRule type="containsText" dxfId="22" priority="15" operator="containsText" text="get approval">
       <formula>NOT(ISERROR(SEARCH("get approval",E4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J21">
-    <cfRule type="cellIs" dxfId="20" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="17" operator="equal">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J34">
-    <cfRule type="cellIs" dxfId="19" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="7" operator="equal">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N21">
-    <cfRule type="expression" dxfId="18" priority="18">
+    <cfRule type="expression" dxfId="19" priority="18">
       <formula>J21=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N34">
-    <cfRule type="expression" dxfId="17" priority="8">
+    <cfRule type="expression" dxfId="18" priority="8">
       <formula>J34=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O21">
-    <cfRule type="expression" dxfId="16" priority="19">
+    <cfRule type="expression" dxfId="17" priority="19">
       <formula>J21=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O22:O30">
-    <cfRule type="cellIs" dxfId="15" priority="11" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="16" priority="11" operator="lessThanOrEqual">
       <formula>0.15</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="12" operator="containsText" text="get approval">
+    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="get approval">
       <formula>NOT(ISERROR(SEARCH("get approval",O22)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O34">
-    <cfRule type="expression" dxfId="13" priority="9">
+    <cfRule type="expression" dxfId="14" priority="9">
       <formula>J34=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O35:O42">
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThanOrEqual">
       <formula>0.15</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="get approval">
+    <cfRule type="containsText" dxfId="12" priority="6" operator="containsText" text="get approval">
       <formula>NOT(ISERROR(SEARCH("get approval",O35)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P15">
-    <cfRule type="containsText" dxfId="10" priority="13" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="11" priority="13" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="14" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="10" priority="14" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P15)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3593,10 +3631,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C57D610-A502-44A5-B585-E13275E054BF}">
-  <dimension ref="A1:X3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:24" s="13" customFormat="1" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" s="13" customFormat="1" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3670,7 +3708,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24" s="15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
         <v>24</v>
       </c>
@@ -3681,7 +3719,7 @@
         <v>26</v>
       </c>
       <c r="D2" s="14" t="str">
-        <f t="shared" ref="D2:D3" si="0">B2&amp;C2</f>
+        <f t="shared" ref="D2:D11" si="0">B2&amp;C2</f>
         <v>Z209BGP</v>
       </c>
       <c r="E2" s="15" t="s">
@@ -3730,7 +3768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" s="15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>24</v>
       </c>
@@ -3750,7 +3788,7 @@
       <c r="F3" s="14">
         <v>3</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="148">
         <v>2</v>
       </c>
       <c r="H3" s="17">
@@ -3790,9 +3828,273 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z409BGP</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="14">
+        <v>4</v>
+      </c>
+      <c r="G4" s="148">
+        <v>3</v>
+      </c>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="18"/>
+    </row>
+    <row r="5" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z509BGP</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="14">
+        <v>5</v>
+      </c>
+      <c r="G5" s="148">
+        <v>4</v>
+      </c>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="17"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="18"/>
+    </row>
+    <row r="6" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z609BGP</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="14">
+        <v>6</v>
+      </c>
+      <c r="G6" s="148">
+        <v>5</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="18"/>
+    </row>
+    <row r="7" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z209BMP</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="14">
+        <v>2</v>
+      </c>
+      <c r="G7" s="148">
+        <v>1</v>
+      </c>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="17"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="18"/>
+    </row>
+    <row r="8" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z309BMP</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="14">
+        <v>3</v>
+      </c>
+      <c r="G8" s="148">
+        <v>2</v>
+      </c>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="17"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="18"/>
+    </row>
+    <row r="9" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z409BMP</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="14">
+        <v>4</v>
+      </c>
+      <c r="G9" s="148">
+        <v>3</v>
+      </c>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="18"/>
+    </row>
+    <row r="10" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z509BMP</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="14">
+        <v>5</v>
+      </c>
+      <c r="G10" s="148">
+        <v>4</v>
+      </c>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="18"/>
+    </row>
+    <row r="11" spans="1:24" s="15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Z609BMP</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="14">
+        <v>6</v>
+      </c>
+      <c r="G11" s="148">
+        <v>5</v>
+      </c>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="17"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="18"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:D3">
-    <cfRule type="duplicateValues" dxfId="8" priority="16"/>
+  <conditionalFormatting sqref="D1:D11">
+    <cfRule type="duplicateValues" dxfId="9" priority="17"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -3802,16 +4104,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94960742-E285-473C-8C0F-56F7DCDD67D8}">
   <dimension ref="A1:U5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="15.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="1" max="2" width="15.109375" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="116" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="116" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="105" t="s">
         <v>0</v>
       </c>
@@ -3876,7 +4178,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:21" s="116" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" s="116" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="117" t="s">
         <v>24</v>
       </c>
@@ -3918,7 +4220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="129" t="s">
         <v>24</v>
       </c>
@@ -3960,7 +4262,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="129" t="s">
         <v>24</v>
       </c>
@@ -4002,7 +4304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="129" t="s">
         <v>24</v>
       </c>
@@ -4046,20 +4348,20 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B5">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:E2">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E5">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
Remove overview and total information + add option to choose between signal power and E&A option in terms of price break
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Example PL.xlsx
+++ b/Example PL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\niels\VSC_Projects\Custom-Odoo\odoo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DD5759-A4A2-48AF-8BCA-72987A7A4A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E087CCE9-F908-4BD3-8CC9-4A3A93242278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0175591F-D8A5-4571-8C6F-C92C3EBD14E9}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="13896" xr2:uid="{0175591F-D8A5-4571-8C6F-C92C3EBD14E9}"/>
   </bookViews>
   <sheets>
     <sheet name="QUOTE" sheetId="3" r:id="rId1"/>
@@ -1641,6 +1641,9 @@
     <xf numFmtId="2" fontId="0" fillId="18" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1680,9 +1683,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1690,17 +1690,7 @@
     <cellStyle name="Komma 2" xfId="2" xr:uid="{CF877343-7E00-44C8-89FB-F4DA51A7E72B}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="24">
     <dxf>
       <font>
         <color rgb="FF9C6500"/>
@@ -2623,20 +2613,20 @@
     </row>
     <row r="14" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C14" s="43"/>
-      <c r="D14" s="138" t="s">
+      <c r="D14" s="139" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="139"/>
-      <c r="F14" s="139"/>
-      <c r="G14" s="139"/>
-      <c r="H14" s="139"/>
-      <c r="I14" s="139"/>
-      <c r="J14" s="139"/>
-      <c r="K14" s="139"/>
-      <c r="L14" s="139"/>
-      <c r="M14" s="140"/>
-      <c r="N14" s="140"/>
-      <c r="O14" s="140"/>
+      <c r="E14" s="140"/>
+      <c r="F14" s="140"/>
+      <c r="G14" s="140"/>
+      <c r="H14" s="140"/>
+      <c r="I14" s="140"/>
+      <c r="J14" s="140"/>
+      <c r="K14" s="140"/>
+      <c r="L14" s="140"/>
+      <c r="M14" s="141"/>
+      <c r="N14" s="141"/>
+      <c r="O14" s="141"/>
       <c r="P14" s="44" t="s">
         <v>50</v>
       </c>
@@ -2647,17 +2637,17 @@
       <c r="D15" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="141"/>
-      <c r="F15" s="141"/>
-      <c r="G15" s="141"/>
-      <c r="H15" s="141"/>
-      <c r="I15" s="141"/>
-      <c r="J15" s="141"/>
-      <c r="K15" s="141"/>
-      <c r="L15" s="141"/>
-      <c r="M15" s="142"/>
-      <c r="N15" s="142"/>
-      <c r="O15" s="142"/>
+      <c r="E15" s="142"/>
+      <c r="F15" s="142"/>
+      <c r="G15" s="142"/>
+      <c r="H15" s="142"/>
+      <c r="I15" s="142"/>
+      <c r="J15" s="142"/>
+      <c r="K15" s="142"/>
+      <c r="L15" s="142"/>
+      <c r="M15" s="143"/>
+      <c r="N15" s="143"/>
+      <c r="O15" s="143"/>
       <c r="P15" s="47" t="s">
         <v>52</v>
       </c>
@@ -2668,17 +2658,17 @@
       <c r="D16" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="142"/>
-      <c r="F16" s="143"/>
-      <c r="G16" s="143"/>
-      <c r="H16" s="143"/>
-      <c r="I16" s="143"/>
-      <c r="J16" s="143"/>
-      <c r="K16" s="143"/>
-      <c r="L16" s="143"/>
-      <c r="M16" s="143"/>
-      <c r="N16" s="143"/>
-      <c r="O16" s="144"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="144"/>
+      <c r="H16" s="144"/>
+      <c r="I16" s="144"/>
+      <c r="J16" s="144"/>
+      <c r="K16" s="144"/>
+      <c r="L16" s="144"/>
+      <c r="M16" s="144"/>
+      <c r="N16" s="144"/>
+      <c r="O16" s="145"/>
       <c r="P16" s="49" t="s">
         <v>54</v>
       </c>
@@ -2689,17 +2679,17 @@
       <c r="D17" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="145"/>
-      <c r="G17" s="145"/>
-      <c r="H17" s="145"/>
-      <c r="I17" s="145"/>
-      <c r="J17" s="145"/>
-      <c r="K17" s="145"/>
-      <c r="L17" s="145"/>
-      <c r="M17" s="146"/>
-      <c r="N17" s="146"/>
-      <c r="O17" s="146"/>
+      <c r="E17" s="146"/>
+      <c r="F17" s="146"/>
+      <c r="G17" s="146"/>
+      <c r="H17" s="146"/>
+      <c r="I17" s="146"/>
+      <c r="J17" s="146"/>
+      <c r="K17" s="146"/>
+      <c r="L17" s="146"/>
+      <c r="M17" s="147"/>
+      <c r="N17" s="147"/>
+      <c r="O17" s="147"/>
       <c r="P17" s="51"/>
       <c r="Q17" s="52" t="str" cm="1">
         <f t="array" ref="Q17">IF(P17&lt;&gt;"",Lastmodified(P17),"")</f>
@@ -2832,8 +2822,7 @@
         <v>10</v>
       </c>
       <c r="K22" s="83">
-        <f>(F22*$H$4)+H22+I22</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" s="82">
         <f>$G$4</f>
@@ -2841,15 +2830,15 @@
       </c>
       <c r="M22" s="84">
         <f>VLOOKUP(L22,MOQ_PUR_SALES_FACTOR,IF(J21=$I$3,3,IF(J21=$J$3,4,IF(J21=$K$3,5,""))),FALSE)*K22</f>
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="N22" s="85">
         <f>L22*M22</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="O22" s="86">
         <f t="shared" ref="O22:O29" si="0">IF($P$17="",IF(VLOOKUP(C22,$C$4:$E$11,2,FALSE)&gt;$D$12,ROUND(M22,2)&amp;" &gt; Get approval",M22),M22)</f>
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="P22" s="87"/>
     </row>
@@ -3133,21 +3122,21 @@
     <row r="31" spans="2:17" s="42" customFormat="1" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B31" s="123"/>
       <c r="C31" s="124"/>
-      <c r="D31" s="147" t="s">
+      <c r="D31" s="148" t="s">
         <v>88</v>
       </c>
-      <c r="E31" s="147"/>
-      <c r="F31" s="147"/>
-      <c r="G31" s="147"/>
-      <c r="H31" s="147"/>
-      <c r="I31" s="147"/>
-      <c r="J31" s="147"/>
-      <c r="K31" s="147"/>
-      <c r="L31" s="147"/>
-      <c r="M31" s="147"/>
-      <c r="N31" s="147"/>
-      <c r="O31" s="147"/>
-      <c r="P31" s="147"/>
+      <c r="E31" s="148"/>
+      <c r="F31" s="148"/>
+      <c r="G31" s="148"/>
+      <c r="H31" s="148"/>
+      <c r="I31" s="148"/>
+      <c r="J31" s="148"/>
+      <c r="K31" s="148"/>
+      <c r="L31" s="148"/>
+      <c r="M31" s="148"/>
+      <c r="N31" s="148"/>
+      <c r="O31" s="148"/>
+      <c r="P31" s="148"/>
     </row>
     <row r="32" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="33" spans="2:16" s="42" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3545,71 +3534,71 @@
     <mergeCell ref="D31:P31"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:P1">
-    <cfRule type="expression" dxfId="24" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="10" stopIfTrue="1">
       <formula>N("_PMRH")=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4:D11">
-    <cfRule type="cellIs" dxfId="23" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="22" priority="16" operator="greaterThan">
       <formula>$D$12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E4:E11">
-    <cfRule type="containsText" dxfId="22" priority="15" operator="containsText" text="get approval">
+    <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="get approval">
       <formula>NOT(ISERROR(SEARCH("get approval",E4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J21">
-    <cfRule type="cellIs" dxfId="21" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="17" operator="equal">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J34">
-    <cfRule type="cellIs" dxfId="20" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="7" operator="equal">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N21">
-    <cfRule type="expression" dxfId="19" priority="18">
+    <cfRule type="expression" dxfId="18" priority="18">
       <formula>J21=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N34">
-    <cfRule type="expression" dxfId="18" priority="8">
+    <cfRule type="expression" dxfId="17" priority="8">
       <formula>J34=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O21">
-    <cfRule type="expression" dxfId="17" priority="19">
+    <cfRule type="expression" dxfId="16" priority="19">
       <formula>J21=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O22:O30">
-    <cfRule type="cellIs" dxfId="16" priority="11" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="15" priority="11" operator="lessThanOrEqual">
       <formula>0.15</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="get approval">
+    <cfRule type="containsText" dxfId="14" priority="12" operator="containsText" text="get approval">
       <formula>NOT(ISERROR(SEARCH("get approval",O22)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O34">
-    <cfRule type="expression" dxfId="14" priority="9">
+    <cfRule type="expression" dxfId="13" priority="9">
       <formula>J34=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O35:O42">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="12" priority="5" operator="lessThanOrEqual">
       <formula>0.15</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="6" operator="containsText" text="get approval">
+    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="get approval">
       <formula>NOT(ISERROR(SEARCH("get approval",O35)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P15">
-    <cfRule type="containsText" dxfId="11" priority="13" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="10" priority="13" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="14" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="9" priority="14" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P15)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3788,7 +3777,7 @@
       <c r="F3" s="14">
         <v>3</v>
       </c>
-      <c r="G3" s="148">
+      <c r="G3" s="138">
         <v>2</v>
       </c>
       <c r="H3" s="17">
@@ -3848,7 +3837,7 @@
       <c r="F4" s="14">
         <v>4</v>
       </c>
-      <c r="G4" s="148">
+      <c r="G4" s="138">
         <v>3</v>
       </c>
       <c r="H4" s="17"/>
@@ -3881,7 +3870,7 @@
       <c r="F5" s="14">
         <v>5</v>
       </c>
-      <c r="G5" s="148">
+      <c r="G5" s="138">
         <v>4</v>
       </c>
       <c r="H5" s="17"/>
@@ -3914,7 +3903,7 @@
       <c r="F6" s="14">
         <v>6</v>
       </c>
-      <c r="G6" s="148">
+      <c r="G6" s="138">
         <v>5</v>
       </c>
       <c r="H6" s="17"/>
@@ -3947,7 +3936,7 @@
       <c r="F7" s="14">
         <v>2</v>
       </c>
-      <c r="G7" s="148">
+      <c r="G7" s="138">
         <v>1</v>
       </c>
       <c r="H7" s="17"/>
@@ -3980,7 +3969,7 @@
       <c r="F8" s="14">
         <v>3</v>
       </c>
-      <c r="G8" s="148">
+      <c r="G8" s="138">
         <v>2</v>
       </c>
       <c r="H8" s="17"/>
@@ -4013,7 +4002,7 @@
       <c r="F9" s="14">
         <v>4</v>
       </c>
-      <c r="G9" s="148">
+      <c r="G9" s="138">
         <v>3</v>
       </c>
       <c r="H9" s="17"/>
@@ -4046,7 +4035,7 @@
       <c r="F10" s="14">
         <v>5</v>
       </c>
-      <c r="G10" s="148">
+      <c r="G10" s="138">
         <v>4</v>
       </c>
       <c r="H10" s="17"/>
@@ -4079,7 +4068,7 @@
       <c r="F11" s="14">
         <v>6</v>
       </c>
-      <c r="G11" s="148">
+      <c r="G11" s="138">
         <v>5</v>
       </c>
       <c r="H11" s="17"/>
@@ -4094,7 +4083,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D11">
-    <cfRule type="duplicateValues" dxfId="9" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="17"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -4348,20 +4337,20 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B5">
-    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:E2">
-    <cfRule type="duplicateValues" dxfId="6" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E5">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>

</xml_diff>